<commit_message>
Add new-customer cohort sheets (新規A / 新規B) to tag_x_telesales
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LC8T_集計結果.xlsx
+++ b/LC8T_集計結果.xlsx
@@ -12,6 +12,8 @@
     <sheet name="acts_target_distribution" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="chocosys_to_set_migration" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="taiwan_birth_trend" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="tag_x_telesales_新規A" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="tag_x_telesales_新規B" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1458,49 +1460,377 @@
       <c r="A2" t="n">
         <v>2018</v>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
         <v>2019</v>
       </c>
-      <c r="B3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
         <v>2020</v>
       </c>
-      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
         <v>2021</v>
       </c>
-      <c r="B5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
         <v>2022</v>
       </c>
-      <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
         <v>2023</v>
       </c>
-      <c r="B7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
         <v>2024</v>
       </c>
-      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
         <v>2025</v>
       </c>
-      <c r="B9" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>標籤数区分</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>客戶数</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>接通客戶数</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>接通率</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>承諾客戶数</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>承諾率</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>60日内成交客戶数</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>成交率</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>157</v>
+      </c>
+      <c r="C2" t="n">
+        <v>92</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="E2" t="n">
+        <v>23</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.293</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>15679</v>
+      </c>
+      <c r="C3" t="n">
+        <v>6661</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.425</v>
+      </c>
+      <c r="E3" t="n">
+        <v>916</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.138</v>
+      </c>
+      <c r="G3" t="n">
+        <v>935</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1981</v>
+      </c>
+      <c r="C4" t="n">
+        <v>711</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.359</v>
+      </c>
+      <c r="E4" t="n">
+        <v>43</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G4" t="n">
+        <v>43</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>6+</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>9814</v>
+      </c>
+      <c r="C5" t="n">
+        <v>3910</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.398</v>
+      </c>
+      <c r="E5" t="n">
+        <v>365</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.093</v>
+      </c>
+      <c r="G5" t="n">
+        <v>426</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.109</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>標籤数区分</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>客戶数</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>接通客戶数</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>接通率</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>承諾客戶数</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>承諾率</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>60日内成交客戶数</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>成交率</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>258</v>
+      </c>
+      <c r="C2" t="n">
+        <v>170</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="E2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="G2" t="n">
+        <v>47</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.276</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4762</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2403</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.505</v>
+      </c>
+      <c r="E3" t="n">
+        <v>457</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="G3" t="n">
+        <v>457</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>409</v>
+      </c>
+      <c r="C4" t="n">
+        <v>117</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.286</v>
+      </c>
+      <c r="E4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.043</v>
+      </c>
+      <c r="G4" t="n">
+        <v>7</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>6+</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4717</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1869</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.396</v>
+      </c>
+      <c r="E5" t="n">
+        <v>226</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="G5" t="n">
+        <v>279</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.149</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add tag-quality cohort sheets (行為件数 / 行為x興趣 cross)
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LC8T_集計結果.xlsx
+++ b/LC8T_集計結果.xlsx
@@ -14,6 +14,8 @@
     <sheet name="taiwan_birth_trend" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="tag_x_telesales_新規A" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="tag_x_telesales_新規B" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="tag_type_行為_x_telesales" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="tag_type_行為x興趣_cross" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1835,4 +1837,365 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>行為タグ件数</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>客戶数</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>接通客戶数</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>接通率</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>承諾客戶数</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>承諾率</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>60日内成交客戶数</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>成交率</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>269</v>
+      </c>
+      <c r="C2" t="n">
+        <v>172</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.639</v>
+      </c>
+      <c r="E2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.233</v>
+      </c>
+      <c r="G2" t="n">
+        <v>48</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.279</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>25489</v>
+      </c>
+      <c r="C3" t="n">
+        <v>12102</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.475</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2135</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.176</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2151</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.178</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2355</v>
+      </c>
+      <c r="C4" t="n">
+        <v>890</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.378</v>
+      </c>
+      <c r="E4" t="n">
+        <v>83</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.093</v>
+      </c>
+      <c r="G4" t="n">
+        <v>93</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.104</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>10398</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4444</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.427</v>
+      </c>
+      <c r="E5" t="n">
+        <v>520</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.117</v>
+      </c>
+      <c r="G5" t="n">
+        <v>611</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.137</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>行為系タグ</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>興趣系タグ</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>客戶数</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>接通客戶数</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>接通率</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>承諾客戶数</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>承諾率</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>60日内成交客戶数</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>成交率</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>なし</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>なし</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>269</v>
+      </c>
+      <c r="D2" t="n">
+        <v>172</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.639</v>
+      </c>
+      <c r="F2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.233</v>
+      </c>
+      <c r="H2" t="n">
+        <v>48</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.279</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>なし</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>なし</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>38049</v>
+      </c>
+      <c r="D4" t="n">
+        <v>17345</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.456</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2725</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.157</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2835</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.163</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>あり</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>193</v>
+      </c>
+      <c r="D5" t="n">
+        <v>91</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.472</v>
+      </c>
+      <c r="F5" t="n">
+        <v>13</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.143</v>
+      </c>
+      <c r="H5" t="n">
+        <v>20</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>